<commit_message>
Benchmark test case result
</commit_message>
<xml_diff>
--- a/tests/Performans Analizi Raporu Taslağı.xlsx
+++ b/tests/Performans Analizi Raporu Taslağı.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahsen.Aslan\Documents\GitHub\distributed-service-dependency-analysis\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0254D29D-DACA-4A2B-B2C4-952CCAAD3C3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B6F1E4-B4E5-4ADA-BF1C-52806F18F3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="1755" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Performans Analizi Raporu Tasla" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,60 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="4">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="4">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>Test ID</t>
   </si>
@@ -89,9 +141,6 @@
     <t>Test Senaryosu</t>
   </si>
   <si>
-    <t>N (Döngü)</t>
-  </si>
-  <si>
     <t>Average (ms)</t>
   </si>
   <si>
@@ -101,12 +150,6 @@
     <t>Max (ms)</t>
   </si>
   <si>
-    <t>Std. Dev (ms)</t>
-  </si>
-  <si>
-    <t>Throughput (TPS)</t>
-  </si>
-  <si>
     <t>Error (%)</t>
   </si>
   <si>
@@ -123,6 +166,25 @@
   </si>
   <si>
     <t>50 Users, 30 Ramp-up, 1 Loop</t>
+  </si>
+  <si>
+    <t>TC-01 senaryosu için yapılan Apache Benchmark doğrulaması, JMeter ile elde edilen verilerle tutarlılık göstermektedir. JMeter üzerinde elde edilen gecikme değerleri, arayüz yükü (GUI overhead) hesaba katıldığında, 'ab' aracı ile elde edilen 10.83 ms'lik saf gecikme değeriyle korelasyon sağlamaktadır. Bu durum, ölçüm metodolojisinin güvenilirliğini kanıtlamaktadır.</t>
+  </si>
+  <si>
+    <t>TC-02 sonuçları, servis odaklı mimarilerde dış bağımlılıkların performans üzerindeki etkisinin doğrusal değil, katlanarak arttığını göstermektedir. Sistemin 'Throughput' değerindeki bu dramatik düşüş, servis tasarımında asenkron iletişim veya önbellekleme (caching) gibi optimizasyonların neden kritik olduğunu sayısal olarak ortaya koymaktadır.</t>
+  </si>
+  <si>
+    <t>TC-03 verileri göstermektedir ki; bir servisin toplam performansı, en yavaş bileşeni olan dış bağımlılık süresi tarafından domine edilmektedir. İşlemci yoğunluklu görevler (CPU Bound), ağ gecikmesinin (I/O Bound) yüksek olduğu senaryolarda toplam süreyi marjinal olarak etkilese de, saniyedeki toplam işlem kapasitesini (Throughput) taban seviyelerde sabitlemektedir.</t>
+  </si>
+  <si>
+    <t>TC-04 senaryosu, dağıtık sistemlerde 'istikrarsız dış bağımlılık' (Unstable Dependency) durumunu simüle etmektedir. Test sonuçlarında görülen 0.66 RPS değeri, sistemin işleme kapasitesinin (Throughput) dış servisteki gecikme süresine doğrudan bağımlı olduğunu kanıtlamaktadır.
+Analiz edilen verilerde, ortalama yanıt süresi 3026 ms iken, medyan değerin 5008 ms olması, sistemdeki gecikmenin homojen olmadığını, belirli bir olasılık dahilinde gerçekleştiğini göstermektedir. Buna rağmen 'Failed Requests: 0' sonucu, sistemin uzun süreli beklemelere karşı dirençli olduğunu ve hata vermeden süreci sonlandırabildiğini (Resilience) belgelemektedir. Bu bulgu, servis tasarımında 'Timeout' ve 'Retry' mekanizmalarının performans maliyetini belirlemek açısından kritik bir veridir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İstek Sayısı </t>
+  </si>
+  <si>
+    <t>Throughput (RPS)</t>
   </si>
 </sst>
 </file>
@@ -174,11 +236,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -194,6 +261,85 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -405,7 +551,7 @@
     <col min="4" max="4" width="53.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" ht="12.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -419,7 +565,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" ht="12.75">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -433,7 +579,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" ht="12.75">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -447,7 +593,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" ht="12.75">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -461,7 +607,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" ht="12.75">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -477,13 +623,13 @@
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
         <v>19</v>
@@ -499,14 +645,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" customWidth="1"/>
+    <col min="7" max="7" width="23.42578125" customWidth="1"/>
+    <col min="9" max="9" width="42.7109375" customWidth="1"/>
+    <col min="10" max="10" width="66.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11" ht="12.75">
       <c r="A1" s="2" t="s">
         <v>20</v>
       </c>
@@ -514,28 +662,25 @@
         <v>21</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+    </row>
+    <row r="2" spans="1:11" ht="147.75" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -543,33 +688,64 @@
         <v>5</v>
       </c>
       <c r="C2" s="2">
-        <v>30</v>
-      </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9">
+        <v>1000</v>
+      </c>
+      <c r="D2" s="2">
+        <v>10.83</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2">
+        <v>215</v>
+      </c>
+      <c r="G2">
+        <v>923.33</v>
+      </c>
+      <c r="H2" s="6">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="176.25" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2">
-        <v>30</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="1:9">
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>448.91</v>
+      </c>
+      <c r="E3" s="2">
+        <v>221</v>
+      </c>
+      <c r="F3">
+        <v>742</v>
+      </c>
+      <c r="G3" s="2">
+        <v>11.14</v>
+      </c>
+      <c r="H3" s="5">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" ht="102">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -577,31 +753,61 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>30</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9">
+        <v>100</v>
+      </c>
+      <c r="D4">
+        <v>3026.39</v>
+      </c>
+      <c r="E4" s="2">
+        <v>119</v>
+      </c>
+      <c r="F4" s="2">
+        <v>798</v>
+      </c>
+      <c r="G4" s="2">
+        <v>12.6</v>
+      </c>
+      <c r="H4" s="6">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="229.5">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2">
-        <v>30</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+        <v>100</v>
+      </c>
+      <c r="D5" s="2">
+        <v>3026.39</v>
+      </c>
+      <c r="E5" s="2">
+        <v>6</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5024</v>
+      </c>
+      <c r="G5" s="2">
+        <v>66</v>
+      </c>
+      <c r="H5" s="6">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Rapor yazmak için test case baştan olluşturuldu
</commit_message>
<xml_diff>
--- a/tests/Performans Analizi Raporu Taslağı.xlsx
+++ b/tests/Performans Analizi Raporu Taslağı.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahsen.Aslan\Documents\GitHub\distributed-service-dependency-analysis\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B6F1E4-B4E5-4ADA-BF1C-52806F18F3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A62FB9E-515C-465A-AA14-905D517B8EEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Performans Analizi Raporu Tasla" sheetId="1" r:id="rId1"/>
     <sheet name="Senaryo" sheetId="2" r:id="rId2"/>
+    <sheet name="08.04.2026-Benchmark Tekrar" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -25,7 +27,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="4">
+  <futureMetadata name="XLRICHVALUE" count="11">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -54,8 +56,57 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="7"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="9"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="10"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="4">
+  <valueMetadata count="11">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -67,13 +118,34 @@
     </bk>
     <bk>
       <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+    <bk>
+      <rc t="1" v="7"/>
+    </bk>
+    <bk>
+      <rc t="1" v="8"/>
+    </bk>
+    <bk>
+      <rc t="1" v="9"/>
+    </bk>
+    <bk>
+      <rc t="1" v="10"/>
     </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="88">
   <si>
     <t>Test ID</t>
   </si>
@@ -185,13 +257,178 @@
   </si>
   <si>
     <t>Throughput (RPS)</t>
+  </si>
+  <si>
+    <t>Test Senaryosu Adı</t>
+  </si>
+  <si>
+    <t>İstek Sayısı (n)</t>
+  </si>
+  <si>
+    <t>Eşzamanlılık (c)</t>
+  </si>
+  <si>
+    <t>Ortalama Yanıt (ms)</t>
+  </si>
+  <si>
+    <t>P99 Gecikme (ms)</t>
+  </si>
+  <si>
+    <t>Akademik Yorum ve Analiz</t>
+  </si>
+  <si>
+    <t>Herhangi bir dış bağımlılık olmadan Gateway'in saf hızı.</t>
+  </si>
+  <si>
+    <t>Sistemin temel kapasitesi oldukça yüksektir. Gecikme minimum düzeyde olup referans noktasıdır.</t>
+  </si>
+  <si>
+    <t>Level 1 (I/O)</t>
+  </si>
+  <si>
+    <t>Dış servisten (API) veri çekme sürecindeki ağ gecikmesi.</t>
+  </si>
+  <si>
+    <t>Sadece bir dış bağımlılık eklenmesi, yanıt süresini Baseline'a göre yaklaşık 56 kat artırmıştır.</t>
+  </si>
+  <si>
+    <t>Veri çekme sonrası SHA256 şifreleme ve Sort işlemi yükü.</t>
+  </si>
+  <si>
+    <t>CPU yükü, I/O bekleme süresiyle asenkron yönetildiği için toplam süreyi TC-02'ye göre radikal artırmamıştır.</t>
+  </si>
+  <si>
+    <t>Resilience (Kararsız)</t>
+  </si>
+  <si>
+    <t>Dış servisin rastgele gecikmeler (3-7 sn) yarattığı durum.</t>
+  </si>
+  <si>
+    <t>Gecikme değişkenliği (Jitter) en yüksek senaryodur. Sistemin öngörülebilirliği bu noktada kaybolmaktadır.</t>
+  </si>
+  <si>
+    <t>Connection Failure</t>
+  </si>
+  <si>
+    <t>Dış servisin kapalı olması durumundaki hata süresi.</t>
+  </si>
+  <si>
+    <t>Timeout sürelerinin yüksekliği, sistemin 19 saniye boyunca kaynakları boşuna kilitlediğini kanıtlamaktadır.</t>
+  </si>
+  <si>
+    <t>TC-06</t>
+  </si>
+  <si>
+    <t>Large Payload</t>
+  </si>
+  <si>
+    <t>10MB boyutundaki büyük veri transferinin maliyeti.</t>
+  </si>
+  <si>
+    <t>Veri boyutu arttıkça seriştirme ve ağ transfer maliyeti, CPU maliyetinin önüne geçmektedir.</t>
+  </si>
+  <si>
+    <t>TC-07</t>
+  </si>
+  <si>
+    <t>Pool Exhaustion</t>
+  </si>
+  <si>
+    <t>Yoğun istek altında bağlantı havuzu (pool) yönetimi.</t>
+  </si>
+  <si>
+    <t>Eşzamanlılık arttığında bağlantı havuzundaki beklemeler darboğaza (bottleneck) yol açmaktadır.</t>
+  </si>
+  <si>
+    <t>TC-08</t>
+  </si>
+  <si>
+    <t>Error Burst</t>
+  </si>
+  <si>
+    <t>Arka arkaya gelen 500 (Internal Server Error) yanıtları.</t>
+  </si>
+  <si>
+    <t>Hata yönetimi süreçlerinin (Exception handling) sistem performansına ek yük getirdiği gözlemlenmiştir.</t>
+  </si>
+  <si>
+    <t>Analiz Resmi</t>
+  </si>
+  <si>
+    <t>Örnek Sayısı (# Samples)</t>
+  </si>
+  <si>
+    <t>Throughput (istek/sn)</t>
+  </si>
+  <si>
+    <t>Hata Oranı (%)</t>
+  </si>
+  <si>
+    <t>Dış bağımlılık içermeyen saf Gateway performansı.</t>
+  </si>
+  <si>
+    <t>JMeter ölçümleri, Apache Benchmark sonuçlarıyla tutarlı bir "Baseline" hızı göstermektedir. Sistemin temel gecikmesi ihmal edilebilir düzeydedir.</t>
+  </si>
+  <si>
+    <t>Dış API'den veri çekme (Network Latency).</t>
+  </si>
+  <si>
+    <t>Dış servis çağrısı eklendiğinde yanıt süresinin arttığı, ancak JMeter'ın bu yük altında kararlı (stable) bir performans sergilediği görülmektedir.</t>
+  </si>
+  <si>
+    <t>Veri çekme + SHA256 şifreleme + Sıralama.</t>
+  </si>
+  <si>
+    <t>Karma senaryoda CPU yükü, I/O gecikmesinin üzerine eklenmiş; asenkron yapı sayesinde sistem kapasitesi (Throughput) korunmuştur.</t>
+  </si>
+  <si>
+    <t>Rastgele gecikmeli dış servis simülasyonu.</t>
+  </si>
+  <si>
+    <t>Yanıt süresindeki 1369 ms'lik artış, kararsız bağımlılıkların sistemdeki "Tail Latency" (kuyruk gecikmesi) üzerindeki doğrudan etkisini kanıtlamaktadır.</t>
+  </si>
+  <si>
+    <t>Servis kapalıyken sistemin tepkisi (Timeout).</t>
+  </si>
+  <si>
+    <r>
+      <t>En Kritik Bulgu:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 53 saniyelik ortalama süre, sistemin hata durumunda "fail-fast" yapamadığını ve kaynakları dakikalarca beklettiğini göstermektedir.</t>
+    </r>
+  </si>
+  <si>
+    <t>10MB boyutundaki veri paketinin aktarımı.</t>
+  </si>
+  <si>
+    <t>Veri boyutu arttıkça, serileştirme (serialization) işleminin performansı domine etmeye başladığı ve sürenin saniyeler bazına çıktığı gözlemlenmiştir.</t>
+  </si>
+  <si>
+    <t>Yoğun eşzamanlı istek (Concurrency) testi.</t>
+  </si>
+  <si>
+    <t>Bağlantı havuzu sınırlarına yaklaşıldığında, isteklerin işlenme süresininBaseline'a göre logaritmik olarak arttığı saptanmıştır.</t>
+  </si>
+  <si>
+    <t>Yoğun hata yanıtları (HTTP 500) altında sistem.</t>
+  </si>
+  <si>
+    <t>Hataların hızlı dönmesi beklense de, Exception yönetiminin sistem üzerinde I/O işlemleriyle benzer bir gecikme yükü oluşturduğu saptanmıştır.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -215,6 +452,21 @@
       <color rgb="FF1F1F1F"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -224,10 +476,36 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -236,7 +514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -246,6 +524,24 @@
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -261,6 +557,107 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4097" name="AutoShape 1" descr="Seçilen resim, lightbox'ta gösteriliyor.">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{744B71AB-0B0C-F249-03F3-625F95E4CE13}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13935075" y="7496175"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4098" name="AutoShape 2" descr="Seçilen resim, lightbox'ta gösteriliyor.">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D07117C-C351-E11E-46C1-DB8BBF4C4B2B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13935075" y="7496175"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -304,7 +701,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="11">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -319,6 +716,34 @@
   </rv>
   <rv s="0">
     <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>8</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>9</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>10</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -339,6 +764,13 @@
   <rel r:id="rId2"/>
   <rel r:id="rId3"/>
   <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
+  <rel r:id="rId10"/>
+  <rel r:id="rId11"/>
 </richValueRels>
 </file>
 
@@ -812,4 +1244,558 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DCB86B5-D7F2-442B-8E45-02D21DE2893E}">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" customWidth="1"/>
+    <col min="3" max="3" width="64" customWidth="1"/>
+    <col min="8" max="8" width="21.85546875" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="51.75" thickBot="1">
+      <c r="A1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="208.5" customHeight="1" thickBot="1">
+      <c r="A2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="9">
+        <v>1000</v>
+      </c>
+      <c r="E2" s="9">
+        <v>100</v>
+      </c>
+      <c r="F2" s="7">
+        <v>7.99</v>
+      </c>
+      <c r="G2" s="7">
+        <v>1251.52</v>
+      </c>
+      <c r="H2" s="9">
+        <v>17</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="181.5" customHeight="1" thickBot="1">
+      <c r="A3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="9">
+        <v>100</v>
+      </c>
+      <c r="E3" s="9">
+        <v>10</v>
+      </c>
+      <c r="F3" s="7">
+        <v>448.91</v>
+      </c>
+      <c r="G3" s="7">
+        <v>22.28</v>
+      </c>
+      <c r="H3" s="9">
+        <v>788</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="179.25" thickBot="1">
+      <c r="A4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="9">
+        <v>100</v>
+      </c>
+      <c r="E4" s="9">
+        <v>10</v>
+      </c>
+      <c r="F4" s="7">
+        <v>396.75</v>
+      </c>
+      <c r="G4" s="7">
+        <v>25.2</v>
+      </c>
+      <c r="H4" s="9">
+        <v>902</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="141.75" customHeight="1" thickBot="1">
+      <c r="A5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="9">
+        <v>50</v>
+      </c>
+      <c r="E5" s="9">
+        <v>5</v>
+      </c>
+      <c r="F5" s="7">
+        <v>3026.39</v>
+      </c>
+      <c r="G5" s="7">
+        <v>1.65</v>
+      </c>
+      <c r="H5" s="9">
+        <v>5024</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="172.5" customHeight="1" thickBot="1">
+      <c r="A6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="9">
+        <v>50</v>
+      </c>
+      <c r="E6" s="9">
+        <v>5</v>
+      </c>
+      <c r="F6" s="7">
+        <v>19301.62</v>
+      </c>
+      <c r="G6" s="7">
+        <v>0.26</v>
+      </c>
+      <c r="H6" s="9">
+        <v>19998</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="J6" t="e" vm="8">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="182.25" customHeight="1" thickBot="1">
+      <c r="A7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="9">
+        <v>50</v>
+      </c>
+      <c r="E7" s="9">
+        <v>5</v>
+      </c>
+      <c r="F7" s="7">
+        <v>8757.25</v>
+      </c>
+      <c r="G7" s="7">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="H7" s="9">
+        <v>9331</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" t="e" vm="9">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="179.25" thickBot="1">
+      <c r="A8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="9">
+        <v>100</v>
+      </c>
+      <c r="E8" s="9">
+        <v>20</v>
+      </c>
+      <c r="F8" s="7">
+        <v>2418.52</v>
+      </c>
+      <c r="G8" s="7">
+        <v>8.27</v>
+      </c>
+      <c r="H8" s="9">
+        <v>3512</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="179.25" thickBot="1">
+      <c r="A9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="9">
+        <v>100</v>
+      </c>
+      <c r="E9" s="9">
+        <v>10</v>
+      </c>
+      <c r="F9" s="7">
+        <v>2376.14</v>
+      </c>
+      <c r="G9" s="7">
+        <v>8.42</v>
+      </c>
+      <c r="H9" s="9">
+        <v>3901</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J9" t="e" vm="11">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BA98021-AB1B-4D7E-9A1A-0A66A8C6D4A7}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="8" max="8" width="105.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="64.5" thickBot="1">
+      <c r="A1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="243" thickBot="1">
+      <c r="A2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="9">
+        <v>30</v>
+      </c>
+      <c r="E2" s="7">
+        <v>5</v>
+      </c>
+      <c r="F2" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="G2" s="12">
+        <v>0</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="243" thickBot="1">
+      <c r="A3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="9">
+        <v>30</v>
+      </c>
+      <c r="E3" s="7">
+        <v>19</v>
+      </c>
+      <c r="F3" s="7">
+        <v>0.71</v>
+      </c>
+      <c r="G3" s="12">
+        <v>0</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="230.25" thickBot="1">
+      <c r="A4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="9">
+        <v>30</v>
+      </c>
+      <c r="E4" s="7">
+        <v>25</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0.71</v>
+      </c>
+      <c r="G4" s="12">
+        <v>0</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="255.75" thickBot="1">
+      <c r="A5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="9">
+        <v>30</v>
+      </c>
+      <c r="E5" s="7">
+        <v>1369</v>
+      </c>
+      <c r="F5" s="7">
+        <v>0.71</v>
+      </c>
+      <c r="G5" s="12">
+        <v>0</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="268.5" thickBot="1">
+      <c r="A6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="9">
+        <v>718</v>
+      </c>
+      <c r="E6" s="7">
+        <v>53186</v>
+      </c>
+      <c r="F6" s="7">
+        <v>0.89</v>
+      </c>
+      <c r="G6" s="12">
+        <v>1</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="243" thickBot="1">
+      <c r="A7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="9">
+        <v>1500</v>
+      </c>
+      <c r="E7" s="7">
+        <v>3179</v>
+      </c>
+      <c r="F7" s="7">
+        <v>5.43</v>
+      </c>
+      <c r="G7" s="12">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="192" thickBot="1">
+      <c r="A8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="9">
+        <v>1500</v>
+      </c>
+      <c r="E8" s="7">
+        <v>2936</v>
+      </c>
+      <c r="F8" s="7">
+        <v>5.42</v>
+      </c>
+      <c r="G8" s="12">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="255.75" thickBot="1">
+      <c r="A9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="9">
+        <v>1500</v>
+      </c>
+      <c r="E9" s="7">
+        <v>2936</v>
+      </c>
+      <c r="F9" s="7">
+        <v>5.43</v>
+      </c>
+      <c r="G9" s="12">
+        <v>1</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tez Yazılanın Hazırlaaması PART 1
</commit_message>
<xml_diff>
--- a/tests/Performans Analizi Raporu Taslağı.xlsx
+++ b/tests/Performans Analizi Raporu Taslağı.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahsen.Aslan\Documents\GitHub\distributed-service-dependency-analysis\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A62FB9E-515C-465A-AA14-905D517B8EEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A53638-B0A3-423C-B4AD-95B2F8353A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Performans Analizi Raporu Tasla" sheetId="1" r:id="rId1"/>
     <sheet name="Senaryo" sheetId="2" r:id="rId2"/>
     <sheet name="08.04.2026-Benchmark Tekrar" sheetId="4" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="5" r:id="rId4"/>
+    <sheet name="08.04.-jmter" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -536,7 +536,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1355,7 +1355,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="179.25" thickBot="1">
+    <row r="4" spans="1:10" ht="51.75" thickBot="1">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
@@ -1483,7 +1483,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="179.25" thickBot="1">
+    <row r="8" spans="1:10" ht="51.75" thickBot="1">
       <c r="A8" s="7" t="s">
         <v>60</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="179.25" thickBot="1">
+    <row r="9" spans="1:10" ht="51.75" thickBot="1">
       <c r="A9" s="7" t="s">
         <v>64</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="243" thickBot="1">
+    <row r="2" spans="1:8" ht="115.5" thickBot="1">
       <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="243" thickBot="1">
+    <row r="3" spans="1:8" ht="102.75" thickBot="1">
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="230.25" thickBot="1">
+    <row r="4" spans="1:8" ht="115.5" thickBot="1">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="255.75" thickBot="1">
+    <row r="5" spans="1:8" ht="90" thickBot="1">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="268.5" thickBot="1">
+    <row r="6" spans="1:8" ht="102.75" thickBot="1">
       <c r="A6" s="7" t="s">
         <v>28</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="243" thickBot="1">
+    <row r="7" spans="1:8" ht="102.75" thickBot="1">
       <c r="A7" s="7" t="s">
         <v>56</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="192" thickBot="1">
+    <row r="8" spans="1:8" ht="90" thickBot="1">
       <c r="A8" s="7" t="s">
         <v>60</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="255.75" thickBot="1">
+    <row r="9" spans="1:8" ht="90" thickBot="1">
       <c r="A9" s="7" t="s">
         <v>64</v>
       </c>

</xml_diff>